<commit_message>
feat: add severity/probability guide to How To sheet; add ? tooltips to all filters
</commit_message>
<xml_diff>
--- a/sample_input/risk_register.xlsx
+++ b/sample_input/risk_register.xlsx
@@ -75,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -89,6 +89,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -1478,11 +1481,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1565,7 +1568,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Type</t>
@@ -1587,7 +1590,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Title</t>
@@ -1609,7 +1612,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Description</t>
@@ -1631,7 +1634,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Project</t>
@@ -1653,7 +1656,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Severity</t>
@@ -1675,7 +1678,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Impact</t>
@@ -1697,7 +1700,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Probability</t>
@@ -1719,7 +1722,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Status</t>
@@ -1741,7 +1744,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Owner</t>
@@ -1763,7 +1766,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Category</t>
@@ -1785,7 +1788,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Identified Date</t>
@@ -1807,7 +1810,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="30" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Due Date</t>
@@ -1829,7 +1832,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="30" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Last Review</t>
@@ -1851,7 +1854,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Response</t>
@@ -1873,7 +1876,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="30" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Trend</t>
@@ -1895,16 +1898,246 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Severity Levels – Quick Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Example Scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="52" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Severe, potentially irreversible impact on operations, finances, or safety</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Data breach exposing customer PII; complete production outage; regulatory shutdown order</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="52" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Major impact affecting multiple teams or significant business functions</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Key system down for several hours; contract penalty triggered; multi-week schedule slip</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="52" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Significant impact on a team or business area requiring prompt attention</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Single service degraded; compliance gap identified; sprint velocity drop &gt;30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="52" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Moderate impact, manageable within normal operations</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Minor feature delay; minor cost overrun &lt;5%; temporary workaround in place</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="52" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Negligible or cosmetic impact with little business consequence</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Documentation gap; minor UI bug; low-urgency process inefficiency</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Probability Levels – Quick Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Example Scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="52" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>VeryHigh</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Almost certain – expected to occur in most circumstances (&gt;80%)</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Known vulnerability actively exploited in the wild; vendor EOL already passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="52" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Likely – will probably occur in many circumstances (60–80%)</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Dependency upgrade overdue; stakeholder delays are a recurring pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="52" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Possible – might occur at some point (40–60%)</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>New regulation under consultation; third-party SLA borderline performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="52" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Unlikely – could occur but not expected (20–40%)</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Rare edge-case failure mode; low-traffic integration with minor instability history</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="52" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>VeryLow</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Rare – may occur only in exceptional circumstances (&lt;20%)</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Black-swan external event; theoretical attack vector with no known active exploits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="20">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="C43:D43"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="C32:D32"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1997,17 +2230,17 @@
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Q2 Security Audit Passed</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Atlas</t>
         </is>
@@ -2019,17 +2252,17 @@
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Auth CVE Patched Ahead of Schedule</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Atlas</t>
         </is>
@@ -2041,17 +2274,17 @@
       </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Phoenix MVP Delivered On Time</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Phoenix</t>
         </is>
@@ -2063,17 +2296,17 @@
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>2026-04-05</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Orion ETL Reliability Up 18%</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Orion</t>
         </is>

</xml_diff>